<commit_message>
D5 for Table 4 modified to have combinations of ATC IV level instead of single ATC IV level and results based on simulated data updated
</commit_message>
<xml_diff>
--- a/i_test/test_D6_Tabella_4_esenzione_2025/g_output/D6_Table_4_cardiocircolatoria.xlsx
+++ b/i_test/test_D6_Tabella_4_esenzione_2025/g_output/D6_Table_4_cardiocircolatoria.xlsx
@@ -416,22 +416,22 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>3136</t>
+          <t>2439</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>1041</t>
+          <t>815</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>1067</t>
+          <t>796</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>1028</t>
+          <t>828</t>
         </is>
       </c>
     </row>
@@ -443,22 +443,22 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>1.569 (50,0%)</t>
+          <t>1.211 (49,7%)</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>505 (48,5%)</t>
+          <t>397 (48,7%)</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>540 (50,6%)</t>
+          <t>402 (50,5%)</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>524 (51,0%)</t>
+          <t>412 (49,8%)</t>
         </is>
       </c>
     </row>
@@ -470,22 +470,22 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>1.063 (33,9%)</t>
+          <t>843 (34,6%)</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>367 (35,3%)</t>
+          <t>292 (35,8%)</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>357 (33,5%)</t>
+          <t>282 (35,4%)</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>339 (33,0%)</t>
+          <t>269 (32,5%)</t>
         </is>
       </c>
     </row>
@@ -497,22 +497,22 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>1.050 (33,5%)</t>
+          <t>811 (33,3%)</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>328 (31,5%)</t>
+          <t>257 (31,5%)</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>371 (34,8%)</t>
+          <t>265 (33,3%)</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>351 (34,1%)</t>
+          <t>289 (34,9%)</t>
         </is>
       </c>
     </row>
@@ -524,22 +524,22 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>1.023 (32,6%)</t>
+          <t>785 (32,2%)</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>346 (33,2%)</t>
+          <t>266 (32,6%)</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>339 (31,8%)</t>
+          <t>249 (31,3%)</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>338 (32,9%)</t>
+          <t>270 (32,6%)</t>
         </is>
       </c>
     </row>
@@ -551,22 +551,22 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>251 (8,0%)</t>
+          <t>1.614 (66,2%)</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>84 (8,1%)</t>
+          <t>544 (66,7%)</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>83 (7,8%)</t>
+          <t>536 (67,3%)</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>84 (8,2%)</t>
+          <t>534 (64,5%)</t>
         </is>
       </c>
     </row>
@@ -585,22 +585,22 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>A10BD07 1.144 (36,5%)</t>
+          <t>B10AE54 176 (7,2%)</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>A10BD07 400 (38,4%)</t>
+          <t>A10BD09 65 (8,0%)</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>A10AE56 394 (36,9%)</t>
+          <t>D10BK02 59 (7,4%)</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>A10BD09 393 (38,2%)</t>
+          <t>B10AE54 66 (8,0%)</t>
         </is>
       </c>
     </row>
@@ -612,22 +612,22 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>A10BH 1.131 (36,1%)</t>
+          <t>A10BD09 167 (6,8%)</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>A10BH 388 (37,3%)</t>
+          <t>A10BD07 62 (7,6%)</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>A10BK 390 (36,6%)</t>
+          <t>J10BD16 58 (7,3%)</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>A10BH 389 (37,8%)</t>
+          <t>M10BX16 66 (8,0%)</t>
         </is>
       </c>
     </row>
@@ -639,22 +639,22 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>A10BD16 1.101 (35,1%)</t>
+          <t>M10BD10 166 (6,8%)</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>A10BD08 371 (35,6%)</t>
+          <t>J10BD23 61 (7,5%)</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>A10BD15 387 (36,3%)</t>
+          <t>A10BD11 57 (7,2%)</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>A10BD13 373 (36,3%)</t>
+          <t>M10BD16 63 (7,6%)</t>
         </is>
       </c>
     </row>
@@ -666,22 +666,22 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>A10AE56 1.097 (35,0%)</t>
+          <t>J10JE54 162 (6,6%)</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>A10BD21 370 (35,5%)</t>
+          <t>J10JE54 59 (7,2%)</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>A10BD07 385 (36,1%)</t>
+          <t>C10BD21 56 (7,0%)</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>A10BD16 372 (36,2%)</t>
+          <t>B10BD21 63 (7,6%)</t>
         </is>
       </c>
     </row>
@@ -693,22 +693,22 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>A10BD09 1.096 (34,9%)</t>
+          <t>M10BD16 161 (6,6%)</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>A10BD16 370 (35,5%)</t>
+          <t>A10BD16 59 (7,2%)</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>A10BD11 385 (36,1%)</t>
+          <t>C10BD08 55 (6,9%)</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>A10BD20 368 (35,8%)</t>
+          <t>A10BH02 61 (7,4%)</t>
         </is>
       </c>
     </row>
@@ -727,22 +727,22 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>A10BD 3.116 (99,4%)</t>
+          <t>A10BD B10BD C10BD J10BD M10BD 12 (0,5%)</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>A10BD 1.032 (99,1%)</t>
+          <t>A10BD B10BD C10BD J10BD M10BD 5 (0,6%)</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>A10BD 1.064 (99,7%)</t>
+          <t>A10BD B10BD C10BD D10BD J10BD 5 (0,6%)</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>A10BD 1.020 (99,2%)</t>
+          <t>A10BD B10BD C10BD J10BD M10BD 5 (0,6%)</t>
         </is>
       </c>
     </row>
@@ -754,22 +754,22 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>A10AE 1.577 (50,3%)</t>
+          <t>A10BD B10BD C10BD D10BD J10BD M10BD 10 (0,4%)</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>A10AE 529 (50,8%)</t>
+          <t>A10BD B10BD C10BD D10BD J10BD M10BD 4 (0,5%)</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>A10AE 541 (50,7%)</t>
+          <t>A10BD B10BD C10BD D10BD J10BD M10BD 3 (0,4%)</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>A10AE 507 (49,3%)</t>
+          <t>A10BD B10BD C10BD D10BD J10BD M10BD 3 (0,4%)</t>
         </is>
       </c>
     </row>
@@ -781,22 +781,22 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>A10BH 946 (30,2%)</t>
+          <t>A10BD B10BD C10BD D10BD J10BD 9 (0,4%)</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>A10BH 325 (31,2%)</t>
+          <t>A10BD B10BD C10BD D10BD J10BD 3 (0,4%)</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>A10BK 325 (30,5%)</t>
+          <t>B10BD C10BD D10BD J10BD M10BD 3 (0,4%)</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>A10BH 325 (31,6%)</t>
+          <t>B10BJ C10BD D10BD J10BD M10BD 2 (0,2%)</t>
         </is>
       </c>
     </row>
@@ -808,22 +808,22 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>A10BK 924 (29,5%)</t>
+          <t>B10BD C10BD D10BD J10BD M10BD 6 (0,2%)</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>A10BK 299 (28,7%)</t>
+          <t>A10BD B10BD D10BD J10BD M10BD 2 (0,2%)</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>A10BJ 312 (29,2%)</t>
+          <t>A10AE B10BD C10BD D10BD J10BD M10BD 2 (0,3%)</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>A10BK 300 (29,2%)</t>
+          <t>B10BD C10BD D10BD J10BD M10BD 2 (0,2%)</t>
         </is>
       </c>
     </row>
@@ -835,22 +835,22 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>A10BX 892 (28,4%)</t>
+          <t>A10BD B10BD D10BD J10BD M10BD 4 (0,2%)</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>A10BX 294 (28,2%)</t>
+          <t>A10AE A10BD C10BD D10BD J10BD J10JE M10BD 2 (0,2%)</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>A10BX 299 (28,0%)</t>
+          <t>A10AE A10BD B10BD D10BD M10BD 2 (0,3%)</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>A10BX 299 (29,1%)</t>
+          <t>A10BD B10BD C10BD C10BJ D10BD 2 (0,2%)</t>
         </is>
       </c>
     </row>

</xml_diff>